<commit_message>
Se añadieron mensajes de error más descriptivos en el modulo de subir excel
</commit_message>
<xml_diff>
--- a/src/main/resources/test/testFile.xlsx
+++ b/src/main/resources/test/testFile.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10830"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pipe/Documents/vs/sipcommb/Envases-backend/src/main/resources/test/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pipe/Documents/welp/sipcommb/back/TodoEnvasesBack/src/main/resources/test/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03F1D11F-DEC7-E041-9F64-D782CBCFAB91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF62A632-DE02-F947-B508-26E3397D934A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="33600" windowHeight="21000" activeTab="4" xr2:uid="{0BF63B95-FFDE-934E-BB3C-357D74685464}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="33600" windowHeight="18540" activeTab="3" xr2:uid="{0BF63B95-FFDE-934E-BB3C-357D74685464}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="90">
   <si>
     <t>diametro</t>
   </si>
@@ -307,6 +307,9 @@
   </si>
   <si>
     <t xml:space="preserve">Extr. Brisa Marina </t>
+  </si>
+  <si>
+    <t>Aceite Mineral gal 2</t>
   </si>
 </sst>
 </file>
@@ -450,30 +453,28 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="3" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="3" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="3" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="3" fillId="5" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="164" fontId="3" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="3" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="3" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="3" fillId="5" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -831,7 +832,7 @@
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A2" s="6">
+      <c r="A2">
         <v>31</v>
       </c>
       <c r="B2" t="s">
@@ -842,7 +843,7 @@
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A3" s="6">
+      <c r="A3">
         <v>32</v>
       </c>
       <c r="B3" t="s">
@@ -853,7 +854,7 @@
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A4" s="6">
+      <c r="A4">
         <v>33</v>
       </c>
       <c r="B4" t="s">
@@ -864,7 +865,7 @@
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A5" s="6">
+      <c r="A5">
         <v>34</v>
       </c>
       <c r="B5" t="s">
@@ -875,7 +876,7 @@
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A6" s="6">
+      <c r="A6">
         <v>35</v>
       </c>
       <c r="B6" t="s">
@@ -886,7 +887,7 @@
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A7" s="6">
+      <c r="A7">
         <v>12</v>
       </c>
       <c r="B7" t="s">
@@ -897,10 +898,10 @@
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A8" s="8" t="s">
+      <c r="A8" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="B8" s="8" t="s">
+      <c r="B8" s="7" t="s">
         <v>36</v>
       </c>
       <c r="C8" t="s">
@@ -1308,7 +1309,7 @@
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A13" s="7" t="s">
+      <c r="A13" s="6" t="s">
         <v>33</v>
       </c>
       <c r="B13" t="s">
@@ -1340,7 +1341,7 @@
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A14" s="7" t="s">
+      <c r="A14" s="6" t="s">
         <v>34</v>
       </c>
       <c r="B14" t="s">
@@ -1381,602 +1382,600 @@
   <dimension ref="A1:K19"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="2" width="21.6640625" style="12" bestFit="1" customWidth="1"/>
-    <col min="3" max="7" width="10.83203125" style="12"/>
-    <col min="8" max="8" width="12.1640625" style="12" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.83203125" style="12" customWidth="1"/>
-    <col min="10" max="10" width="42.1640625" style="12" customWidth="1"/>
-    <col min="11" max="11" width="41" style="12" bestFit="1" customWidth="1"/>
-    <col min="12" max="16384" width="10.83203125" style="12"/>
+    <col min="1" max="2" width="21.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.1640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.83203125" customWidth="1"/>
+    <col min="10" max="10" width="42.1640625" customWidth="1"/>
+    <col min="11" max="11" width="41" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A1" s="12" t="s">
+      <c r="A1" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="12" t="s">
+      <c r="B1" t="s">
         <v>38</v>
       </c>
-      <c r="C1" s="12" t="s">
+      <c r="C1" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="12" t="s">
+      <c r="D1" t="s">
         <v>11</v>
       </c>
-      <c r="E1" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="F1" s="12" t="s">
+      <c r="E1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F1" t="s">
         <v>13</v>
       </c>
-      <c r="G1" s="12" t="s">
+      <c r="G1" t="s">
         <v>39</v>
       </c>
-      <c r="H1" s="12" t="s">
+      <c r="H1" t="s">
         <v>15</v>
       </c>
-      <c r="I1" s="12" t="s">
+      <c r="I1" t="s">
         <v>17</v>
       </c>
-      <c r="J1" s="12" t="s">
+      <c r="J1" t="s">
         <v>40</v>
       </c>
-      <c r="K1" s="12" t="s">
+      <c r="K1" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A2" s="11" t="s">
+      <c r="A2" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="B2" s="11" t="s">
+      <c r="B2" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="C2" s="12">
-        <v>12</v>
-      </c>
-      <c r="D2" s="13">
+      <c r="C2">
+        <v>12</v>
+      </c>
+      <c r="D2" s="11">
         <v>350</v>
       </c>
-      <c r="E2" s="14">
+      <c r="E2" s="12">
         <v>300</v>
       </c>
-      <c r="F2" s="15">
+      <c r="F2" s="13">
         <v>300</v>
       </c>
-      <c r="G2" s="16">
+      <c r="G2" s="14">
         <v>311</v>
       </c>
-      <c r="H2" s="16">
+      <c r="H2" s="14">
         <v>230</v>
       </c>
-      <c r="I2" s="12">
-        <v>10</v>
-      </c>
-      <c r="K2" s="17" t="s">
+      <c r="I2">
+        <v>10</v>
+      </c>
+      <c r="K2" s="15" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A3" s="11" t="s">
+      <c r="A3" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="B3" s="11" t="s">
+      <c r="B3" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="C3" s="12">
-        <v>12</v>
-      </c>
-      <c r="D3" s="13">
+      <c r="C3">
+        <v>12</v>
+      </c>
+      <c r="D3" s="11">
         <v>250</v>
       </c>
-      <c r="E3" s="14">
+      <c r="E3" s="12">
         <v>200</v>
       </c>
-      <c r="F3" s="15">
+      <c r="F3" s="13">
         <v>185</v>
       </c>
-      <c r="G3" s="16">
+      <c r="G3" s="14">
         <v>160</v>
       </c>
-      <c r="H3" s="16">
+      <c r="H3" s="14">
         <v>4000</v>
       </c>
-      <c r="I3" s="12">
-        <v>10</v>
-      </c>
-      <c r="K3" s="17" t="s">
+      <c r="I3">
+        <v>10</v>
+      </c>
+      <c r="K3" s="15" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A4" s="11" t="s">
+      <c r="A4" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="B4" s="11" t="s">
+      <c r="B4" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="C4" s="12">
-        <v>12</v>
-      </c>
-      <c r="D4" s="13">
+      <c r="C4">
+        <v>12</v>
+      </c>
+      <c r="D4" s="11">
         <v>250</v>
       </c>
-      <c r="E4" s="14">
+      <c r="E4" s="12">
         <v>200</v>
       </c>
-      <c r="F4" s="15">
+      <c r="F4" s="13">
         <v>185</v>
       </c>
-      <c r="G4" s="16">
+      <c r="G4" s="14">
         <v>160</v>
       </c>
-      <c r="H4" s="16">
+      <c r="H4" s="14">
         <v>4000</v>
       </c>
-      <c r="I4" s="12">
-        <v>10</v>
-      </c>
-      <c r="K4" s="17" t="s">
+      <c r="I4">
+        <v>10</v>
+      </c>
+      <c r="K4" s="15" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A5" s="11" t="s">
+      <c r="A5" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="B5" s="11" t="s">
+      <c r="B5" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="C5" s="12">
-        <v>12</v>
-      </c>
-      <c r="D5" s="13">
+      <c r="C5">
+        <v>12</v>
+      </c>
+      <c r="D5" s="11">
         <v>450</v>
       </c>
-      <c r="E5" s="14">
+      <c r="E5" s="12">
         <v>400</v>
       </c>
-      <c r="F5" s="15">
+      <c r="F5" s="13">
         <v>425</v>
       </c>
-      <c r="G5" s="16">
+      <c r="G5" s="14">
         <v>405</v>
       </c>
-      <c r="H5" s="16">
+      <c r="H5" s="14">
         <v>550</v>
       </c>
-      <c r="I5" s="12">
-        <v>10</v>
-      </c>
-      <c r="K5" s="17" t="s">
+      <c r="I5">
+        <v>10</v>
+      </c>
+      <c r="K5" s="15" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A6" s="11" t="s">
+      <c r="A6" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="B6" s="11" t="s">
+      <c r="B6" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="C6" s="12">
-        <v>12</v>
-      </c>
-      <c r="D6" s="13">
+      <c r="C6">
+        <v>12</v>
+      </c>
+      <c r="D6" s="11">
         <v>450</v>
       </c>
-      <c r="E6" s="14">
+      <c r="E6" s="12">
         <v>400</v>
       </c>
-      <c r="F6" s="15">
+      <c r="F6" s="13">
         <v>425</v>
       </c>
-      <c r="G6" s="16">
+      <c r="G6" s="14">
         <v>405</v>
       </c>
-      <c r="H6" s="16">
+      <c r="H6" s="14">
         <v>550</v>
       </c>
-      <c r="I6" s="12">
-        <v>10</v>
-      </c>
-      <c r="K6" s="17" t="s">
+      <c r="I6">
+        <v>10</v>
+      </c>
+      <c r="K6" s="15" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A7" s="11" t="s">
+      <c r="A7" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="B7" s="11" t="s">
+      <c r="B7" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="C7" s="12">
-        <v>12</v>
-      </c>
-      <c r="D7" s="13">
+      <c r="C7">
+        <v>12</v>
+      </c>
+      <c r="D7" s="11">
         <v>300</v>
       </c>
-      <c r="E7" s="14">
+      <c r="E7" s="12">
         <v>250</v>
       </c>
-      <c r="F7" s="15">
+      <c r="F7" s="13">
         <v>235</v>
       </c>
-      <c r="G7" s="16">
+      <c r="G7" s="14">
         <v>215</v>
       </c>
-      <c r="H7" s="16">
+      <c r="H7" s="14">
         <v>3500</v>
       </c>
-      <c r="I7" s="12">
-        <v>10</v>
-      </c>
-      <c r="K7" s="17" t="s">
+      <c r="I7">
+        <v>10</v>
+      </c>
+      <c r="K7" s="15" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A8" s="11" t="s">
+      <c r="A8" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="B8" s="11" t="s">
+      <c r="B8" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="C8" s="12">
-        <v>12</v>
-      </c>
-      <c r="D8" s="13">
+      <c r="C8">
+        <v>12</v>
+      </c>
+      <c r="D8" s="11">
         <v>250</v>
       </c>
-      <c r="E8" s="14">
+      <c r="E8" s="12">
         <v>200</v>
       </c>
-      <c r="F8" s="15">
+      <c r="F8" s="13">
         <v>210</v>
       </c>
-      <c r="G8" s="16">
+      <c r="G8" s="14">
         <v>192</v>
       </c>
-      <c r="H8" s="16">
+      <c r="H8" s="14">
         <v>2600</v>
       </c>
-      <c r="I8" s="12">
-        <v>10</v>
-      </c>
-      <c r="K8" s="17" t="s">
+      <c r="I8">
+        <v>10</v>
+      </c>
+      <c r="K8" s="15" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A9" s="11" t="s">
+      <c r="A9" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="B9" s="11" t="s">
+      <c r="B9" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="C9" s="12">
-        <v>12</v>
-      </c>
-      <c r="D9" s="13">
+      <c r="C9">
+        <v>12</v>
+      </c>
+      <c r="D9" s="11">
         <v>250</v>
       </c>
-      <c r="E9" s="14">
+      <c r="E9" s="12">
         <v>200</v>
       </c>
-      <c r="F9" s="15">
+      <c r="F9" s="13">
         <v>210</v>
       </c>
-      <c r="G9" s="16">
+      <c r="G9" s="14">
         <v>192</v>
       </c>
-      <c r="H9" s="16">
+      <c r="H9" s="14">
         <v>2600</v>
       </c>
-      <c r="I9" s="12">
-        <v>10</v>
-      </c>
-      <c r="K9" s="18" t="s">
+      <c r="I9">
+        <v>10</v>
+      </c>
+      <c r="K9" s="16" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A10" s="11" t="s">
+      <c r="A10" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="B10" s="11" t="s">
+      <c r="B10" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="C10" s="12">
-        <v>12</v>
-      </c>
-      <c r="D10" s="13">
+      <c r="C10">
+        <v>12</v>
+      </c>
+      <c r="D10" s="11">
         <v>300</v>
       </c>
-      <c r="E10" s="14">
+      <c r="E10" s="12">
         <v>250</v>
       </c>
-      <c r="F10" s="15">
+      <c r="F10" s="13">
         <v>210</v>
       </c>
-      <c r="G10" s="16">
+      <c r="G10" s="14">
         <v>192</v>
       </c>
-      <c r="H10" s="16">
+      <c r="H10" s="14">
         <v>1000</v>
       </c>
-      <c r="I10" s="12">
-        <v>10</v>
-      </c>
-      <c r="K10" s="17" t="s">
+      <c r="I10">
+        <v>10</v>
+      </c>
+      <c r="K10" s="15" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A11" s="11" t="s">
+      <c r="A11" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="B11" s="11" t="s">
+      <c r="B11" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="C11" s="12">
-        <v>12</v>
-      </c>
-      <c r="D11" s="13">
+      <c r="C11">
+        <v>12</v>
+      </c>
+      <c r="D11" s="11">
         <v>300</v>
       </c>
-      <c r="E11" s="14">
+      <c r="E11" s="12">
         <v>250</v>
       </c>
-      <c r="F11" s="15">
+      <c r="F11" s="13">
         <v>225</v>
       </c>
-      <c r="G11" s="16">
+      <c r="G11" s="14">
         <v>215</v>
       </c>
-      <c r="H11" s="16">
+      <c r="H11" s="14">
         <v>1000</v>
       </c>
-      <c r="I11" s="12">
-        <v>10</v>
-      </c>
-      <c r="K11" s="17" t="s">
+      <c r="I11">
+        <v>10</v>
+      </c>
+      <c r="K11" s="15" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A12" s="11" t="s">
+      <c r="A12" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="B12" s="11" t="s">
+      <c r="B12" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="C12" s="12">
-        <v>12</v>
-      </c>
-      <c r="D12" s="13">
+      <c r="C12">
+        <v>12</v>
+      </c>
+      <c r="D12" s="11">
         <v>300</v>
       </c>
-      <c r="E12" s="14">
+      <c r="E12" s="12">
         <v>250</v>
       </c>
-      <c r="F12" s="15">
+      <c r="F12" s="13">
         <v>225</v>
       </c>
-      <c r="G12" s="16">
+      <c r="G12" s="14">
         <v>215</v>
       </c>
-      <c r="H12" s="16">
+      <c r="H12" s="14">
         <v>1000</v>
       </c>
-      <c r="I12" s="12">
-        <v>10</v>
-      </c>
-      <c r="K12" s="18" t="s">
+      <c r="I12">
+        <v>10</v>
+      </c>
+      <c r="K12" s="16" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A13" s="11" t="s">
+      <c r="A13" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="B13" s="11" t="s">
+      <c r="B13" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="C13" s="12">
-        <v>12</v>
-      </c>
-      <c r="D13" s="13">
+      <c r="C13">
+        <v>12</v>
+      </c>
+      <c r="D13" s="11">
         <v>200</v>
       </c>
-      <c r="E13" s="14">
+      <c r="E13" s="12">
         <v>150</v>
       </c>
-      <c r="F13" s="15">
+      <c r="F13" s="13">
         <v>160</v>
       </c>
-      <c r="G13" s="16">
+      <c r="G13" s="14">
         <v>122</v>
       </c>
-      <c r="H13" s="16">
+      <c r="H13" s="14">
         <v>1000</v>
       </c>
-      <c r="I13" s="12">
-        <v>10</v>
-      </c>
-      <c r="K13" s="17" t="s">
+      <c r="I13">
+        <v>10</v>
+      </c>
+      <c r="K13" s="15" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A14" s="11" t="s">
+      <c r="A14" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="B14" s="11" t="s">
+      <c r="B14" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="C14" s="12">
-        <v>12</v>
-      </c>
-      <c r="D14" s="13">
+      <c r="C14">
+        <v>12</v>
+      </c>
+      <c r="D14" s="11">
         <v>250</v>
       </c>
-      <c r="E14" s="14">
+      <c r="E14" s="12">
         <v>200</v>
       </c>
-      <c r="F14" s="15">
+      <c r="F14" s="13">
         <v>160</v>
       </c>
-      <c r="G14" s="16">
+      <c r="G14" s="14">
         <v>140</v>
       </c>
-      <c r="H14" s="16">
+      <c r="H14" s="14">
         <v>7000</v>
       </c>
-      <c r="I14" s="12">
-        <v>10</v>
-      </c>
-      <c r="K14" s="18" t="s">
+      <c r="I14">
+        <v>10</v>
+      </c>
+      <c r="K14" s="16" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A15" s="11" t="s">
+      <c r="A15" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="B15" s="11" t="s">
+      <c r="B15" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="C15" s="12">
-        <v>12</v>
-      </c>
-      <c r="D15" s="13">
+      <c r="C15">
+        <v>12</v>
+      </c>
+      <c r="D15" s="11">
         <v>350</v>
       </c>
-      <c r="E15" s="14">
+      <c r="E15" s="12">
         <v>300</v>
       </c>
-      <c r="F15" s="15">
+      <c r="F15" s="13">
         <v>310</v>
       </c>
-      <c r="G15" s="16">
+      <c r="G15" s="14">
         <v>285</v>
       </c>
-      <c r="H15" s="16">
+      <c r="H15" s="14">
         <v>500</v>
       </c>
-      <c r="I15" s="12">
-        <v>10</v>
-      </c>
-      <c r="K15" s="17" t="s">
+      <c r="I15">
+        <v>10</v>
+      </c>
+      <c r="K15" s="15" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A16" s="11" t="s">
+      <c r="A16" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="B16" s="11" t="s">
+      <c r="B16" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="C16" s="12">
-        <v>12</v>
-      </c>
-      <c r="D16" s="13">
+      <c r="C16">
+        <v>12</v>
+      </c>
+      <c r="D16" s="11">
         <v>350</v>
       </c>
-      <c r="E16" s="14">
+      <c r="E16" s="12">
         <v>300</v>
       </c>
-      <c r="F16" s="15">
+      <c r="F16" s="13">
         <v>310</v>
       </c>
-      <c r="G16" s="16">
+      <c r="G16" s="14">
         <v>285</v>
       </c>
-      <c r="H16" s="16">
+      <c r="H16" s="14">
         <v>1000</v>
       </c>
-      <c r="I16" s="12">
-        <v>10</v>
-      </c>
-      <c r="K16" s="17" t="s">
+      <c r="I16">
+        <v>10</v>
+      </c>
+      <c r="K16" s="15" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A17" s="11" t="s">
+      <c r="A17" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="B17" s="11" t="s">
+      <c r="B17" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="C17" s="12">
-        <v>12</v>
-      </c>
-      <c r="D17" s="13">
+      <c r="C17">
+        <v>12</v>
+      </c>
+      <c r="D17" s="11">
         <v>350</v>
       </c>
-      <c r="E17" s="14">
+      <c r="E17" s="12">
         <v>300</v>
       </c>
-      <c r="F17" s="15">
+      <c r="F17" s="13">
         <v>310</v>
       </c>
-      <c r="G17" s="16">
+      <c r="G17" s="14">
         <v>285</v>
       </c>
-      <c r="H17" s="16">
+      <c r="H17" s="14">
         <v>1000</v>
       </c>
-      <c r="I17" s="12">
-        <v>10</v>
-      </c>
-      <c r="K17" s="17" t="s">
+      <c r="I17">
+        <v>10</v>
+      </c>
+      <c r="K17" s="15" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A18" s="11" t="s">
+      <c r="A18" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="B18" s="11" t="s">
+      <c r="B18" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="C18" s="12">
-        <v>12</v>
-      </c>
-      <c r="D18" s="13">
+      <c r="C18">
+        <v>12</v>
+      </c>
+      <c r="D18" s="11">
         <v>400</v>
       </c>
-      <c r="E18" s="14">
+      <c r="E18" s="12">
         <v>350</v>
       </c>
-      <c r="F18" s="15">
+      <c r="F18" s="13">
         <v>335</v>
       </c>
-      <c r="G18" s="16">
+      <c r="G18" s="14">
         <v>320</v>
       </c>
-      <c r="H18" s="16">
+      <c r="H18" s="14">
         <v>800</v>
       </c>
-      <c r="I18" s="12">
-        <v>10</v>
-      </c>
-      <c r="J18" s="17" t="s">
+      <c r="I18">
+        <v>10</v>
+      </c>
+      <c r="J18" s="15" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A19" s="11"/>
-      <c r="B19" s="11"/>
-      <c r="D19" s="13"/>
-      <c r="E19" s="14"/>
-      <c r="F19" s="15"/>
-      <c r="G19" s="16"/>
-      <c r="H19" s="16"/>
+      <c r="A19" s="10"/>
+      <c r="B19" s="10"/>
+      <c r="D19" s="11"/>
+      <c r="E19" s="12"/>
+      <c r="F19" s="13"/>
+      <c r="G19" s="14"/>
+      <c r="H19" s="14"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1985,7 +1984,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{83645BCF-40D5-3E4C-AA9C-7A807E3FA68C}">
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="2" width="23.6640625" bestFit="1" customWidth="1"/>
@@ -2006,13 +2005,13 @@
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A2" s="9" t="s">
+      <c r="A2" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="B2" s="9" t="s">
+      <c r="B2" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="C2" s="10">
+      <c r="C2" s="9">
         <v>96000</v>
       </c>
       <c r="D2">
@@ -2020,13 +2019,13 @@
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A3" s="9" t="s">
+      <c r="A3" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="B3" s="9" t="s">
+      <c r="B3" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="C3" s="10">
+      <c r="C3" s="9">
         <v>50000</v>
       </c>
       <c r="D3">
@@ -2034,13 +2033,13 @@
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A4" s="9" t="s">
+      <c r="A4" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="B4" s="9" t="s">
+      <c r="B4" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="C4" s="10">
+      <c r="C4" s="9">
         <v>466000</v>
       </c>
       <c r="D4">
@@ -2048,13 +2047,13 @@
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A5" s="9" t="s">
+      <c r="A5" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="B5" s="9" t="s">
+      <c r="B5" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="C5" s="10">
+      <c r="C5" s="9">
         <v>12000</v>
       </c>
       <c r="D5">
@@ -2062,13 +2061,13 @@
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A6" s="9" t="s">
+      <c r="A6" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="B6" s="9" t="s">
+      <c r="B6" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="C6" s="10">
+      <c r="C6" s="9">
         <v>20000</v>
       </c>
       <c r="D6">
@@ -2076,13 +2075,13 @@
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A7" s="9" t="s">
+      <c r="A7" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="B7" s="9" t="s">
+      <c r="B7" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="C7" s="10">
+      <c r="C7" s="9">
         <v>35000</v>
       </c>
       <c r="D7">
@@ -2090,13 +2089,13 @@
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A8" s="9" t="s">
+      <c r="A8" s="8" t="s">
         <v>67</v>
       </c>
-      <c r="B8" s="9" t="s">
+      <c r="B8" s="8" t="s">
         <v>67</v>
       </c>
-      <c r="C8" s="10">
+      <c r="C8" s="9">
         <v>68000</v>
       </c>
       <c r="D8">
@@ -2104,13 +2103,13 @@
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A9" s="9" t="s">
+      <c r="A9" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="B9" s="9" t="s">
+      <c r="B9" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="C9" s="10">
+      <c r="C9" s="9">
         <v>133000</v>
       </c>
       <c r="D9">
@@ -2118,13 +2117,13 @@
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A10" s="9" t="s">
+      <c r="A10" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="B10" s="9" t="s">
+      <c r="B10" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="C10" s="10">
+      <c r="C10" s="9">
         <v>23000</v>
       </c>
       <c r="D10">
@@ -2132,13 +2131,13 @@
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A11" s="9" t="s">
+      <c r="A11" s="8" t="s">
         <v>70</v>
       </c>
-      <c r="B11" s="9" t="s">
+      <c r="B11" s="8" t="s">
         <v>70</v>
       </c>
-      <c r="C11" s="10">
+      <c r="C11" s="9">
         <v>13000</v>
       </c>
       <c r="D11">
@@ -2146,13 +2145,13 @@
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A12" s="9" t="s">
+      <c r="A12" s="8" t="s">
         <v>71</v>
       </c>
-      <c r="B12" s="9" t="s">
+      <c r="B12" s="8" t="s">
         <v>71</v>
       </c>
-      <c r="C12" s="10">
+      <c r="C12" s="9">
         <v>7000</v>
       </c>
       <c r="D12">
@@ -2160,13 +2159,13 @@
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A13" s="9" t="s">
+      <c r="A13" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="B13" s="9" t="s">
+      <c r="B13" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="C13" s="10">
+      <c r="C13" s="9">
         <v>139000</v>
       </c>
       <c r="D13">
@@ -2174,13 +2173,13 @@
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A14" s="9" t="s">
+      <c r="A14" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="B14" s="9" t="s">
+      <c r="B14" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="C14" s="10">
+      <c r="C14" s="9">
         <v>71500</v>
       </c>
       <c r="D14">
@@ -2188,17 +2187,31 @@
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A15" s="9" t="s">
+      <c r="A15" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="B15" s="9" t="s">
+      <c r="B15" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="C15" s="10">
+      <c r="C15" s="9">
         <v>43000</v>
       </c>
       <c r="D15">
         <v>10</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A16" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="B16" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="C16" s="9">
+        <v>43000</v>
+      </c>
+      <c r="D16">
+        <v>-10</v>
       </c>
     </row>
   </sheetData>
@@ -2224,25 +2237,25 @@
       <c r="B1" t="s">
         <v>38</v>
       </c>
-      <c r="C1" s="19" t="s">
+      <c r="C1" s="17" t="s">
         <v>80</v>
       </c>
-      <c r="D1" s="19" t="s">
+      <c r="D1" s="17" t="s">
         <v>79</v>
       </c>
-      <c r="E1" s="19" t="s">
+      <c r="E1" s="17" t="s">
         <v>78</v>
       </c>
-      <c r="F1" s="19" t="s">
+      <c r="F1" s="17" t="s">
         <v>77</v>
       </c>
-      <c r="G1" s="19" t="s">
+      <c r="G1" s="17" t="s">
         <v>76</v>
       </c>
-      <c r="H1" s="19" t="s">
+      <c r="H1" s="17" t="s">
         <v>82</v>
       </c>
-      <c r="I1" s="19" t="s">
+      <c r="I1" s="17" t="s">
         <v>81</v>
       </c>
     </row>
@@ -2253,22 +2266,22 @@
       <c r="B2" t="s">
         <v>83</v>
       </c>
-      <c r="C2" s="10">
+      <c r="C2" s="9">
         <v>107000</v>
       </c>
-      <c r="D2" s="10">
+      <c r="D2" s="9">
         <v>55000</v>
       </c>
-      <c r="E2" s="10">
+      <c r="E2" s="9">
         <v>29000</v>
       </c>
-      <c r="F2" s="10">
+      <c r="F2" s="9">
         <v>16000</v>
       </c>
-      <c r="G2" s="10">
+      <c r="G2" s="9">
         <v>9000</v>
       </c>
-      <c r="H2" s="10">
+      <c r="H2" s="9">
         <v>5000</v>
       </c>
       <c r="I2">
@@ -2282,22 +2295,22 @@
       <c r="B3" t="s">
         <v>84</v>
       </c>
-      <c r="C3" s="10">
+      <c r="C3" s="9">
         <v>106000</v>
       </c>
-      <c r="D3" s="10">
+      <c r="D3" s="9">
         <v>54000</v>
       </c>
-      <c r="E3" s="10">
+      <c r="E3" s="9">
         <v>28000</v>
       </c>
-      <c r="F3" s="10">
+      <c r="F3" s="9">
         <v>21000</v>
       </c>
-      <c r="G3" s="10">
+      <c r="G3" s="9">
         <v>11500</v>
       </c>
-      <c r="H3" s="10">
+      <c r="H3" s="9">
         <v>5000</v>
       </c>
       <c r="I3">
@@ -2311,22 +2324,22 @@
       <c r="B4" t="s">
         <v>85</v>
       </c>
-      <c r="C4" s="10">
+      <c r="C4" s="9">
         <v>99000</v>
       </c>
-      <c r="D4" s="10">
+      <c r="D4" s="9">
         <v>51000</v>
       </c>
-      <c r="E4" s="10">
+      <c r="E4" s="9">
         <v>26000</v>
       </c>
-      <c r="F4" s="10">
+      <c r="F4" s="9">
         <v>24000</v>
       </c>
-      <c r="G4" s="10">
+      <c r="G4" s="9">
         <v>13000</v>
       </c>
-      <c r="H4" s="10">
+      <c r="H4" s="9">
         <v>4000</v>
       </c>
       <c r="I4">
@@ -2340,22 +2353,22 @@
       <c r="B5" t="s">
         <v>86</v>
       </c>
-      <c r="C5" s="10">
+      <c r="C5" s="9">
         <v>165000</v>
       </c>
-      <c r="D5" s="10">
+      <c r="D5" s="9">
         <v>84000</v>
       </c>
-      <c r="E5" s="10">
+      <c r="E5" s="9">
         <v>44000</v>
       </c>
-      <c r="F5" s="10">
+      <c r="F5" s="9">
         <v>24000</v>
       </c>
-      <c r="G5" s="10">
+      <c r="G5" s="9">
         <v>13000</v>
       </c>
-      <c r="H5" s="10">
+      <c r="H5" s="9">
         <v>7000</v>
       </c>
       <c r="I5">
@@ -2369,22 +2382,22 @@
       <c r="B6" t="s">
         <v>87</v>
       </c>
-      <c r="C6" s="10">
+      <c r="C6" s="9">
         <v>131000</v>
       </c>
-      <c r="D6" s="10">
+      <c r="D6" s="9">
         <v>67000</v>
       </c>
-      <c r="E6" s="10">
+      <c r="E6" s="9">
         <v>35000</v>
       </c>
-      <c r="F6" s="10">
+      <c r="F6" s="9">
         <v>19000</v>
       </c>
-      <c r="G6" s="10">
+      <c r="G6" s="9">
         <v>10500</v>
       </c>
-      <c r="H6" s="10">
+      <c r="H6" s="9">
         <v>6000</v>
       </c>
       <c r="I6">
@@ -2398,22 +2411,22 @@
       <c r="B7" t="s">
         <v>88</v>
       </c>
-      <c r="C7" s="10">
+      <c r="C7" s="9">
         <v>85000</v>
       </c>
-      <c r="D7" s="10">
+      <c r="D7" s="9">
         <v>43000</v>
       </c>
-      <c r="E7" s="10">
+      <c r="E7" s="9">
         <v>23000</v>
       </c>
-      <c r="F7" s="10">
+      <c r="F7" s="9">
         <v>12000</v>
       </c>
-      <c r="G7" s="10">
+      <c r="G7" s="9">
         <v>7000</v>
       </c>
-      <c r="H7" s="10">
+      <c r="H7" s="9">
         <v>4000</v>
       </c>
       <c r="I7">

</xml_diff>

<commit_message>
Se cambio un poco el excel
</commit_message>
<xml_diff>
--- a/src/main/resources/test/testFile.xlsx
+++ b/src/main/resources/test/testFile.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pipe/Documents/welp/sipcommb/back/TodoEnvasesBack/src/main/resources/test/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF62A632-DE02-F947-B508-26E3397D934A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C16C69E-0C56-304D-93CA-C1EB3F7F0C16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="33600" windowHeight="18540" activeTab="3" xr2:uid="{0BF63B95-FFDE-934E-BB3C-357D74685464}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="33600" windowHeight="21000" activeTab="1" xr2:uid="{0BF63B95-FFDE-934E-BB3C-357D74685464}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,7 @@
     <sheet name="Sheet4" sheetId="4" r:id="rId4"/>
     <sheet name="Sheet5" sheetId="5" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="131">
   <si>
     <t>diametro</t>
   </si>
@@ -310,6 +310,129 @@
   </si>
   <si>
     <t>Aceite Mineral gal 2</t>
+  </si>
+  <si>
+    <t>Pitorro Laboratorio 2</t>
+  </si>
+  <si>
+    <t>Pitorro Laboratorio 3</t>
+  </si>
+  <si>
+    <t>Env. 1000ml Bala Pet Blanco R28</t>
+  </si>
+  <si>
+    <t>Env. 1000ml Bala Pet Fuerte R28</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Env. 1000ml Bala Pet Liviano R28 </t>
+  </si>
+  <si>
+    <t>Env. 1000ml Bala Pet Pesado  R28</t>
+  </si>
+  <si>
+    <t>Tapa 28 Seg. Corta, Tapa Fliptop Cosmet. 28</t>
+  </si>
+  <si>
+    <t>Jarros y tapas de 28</t>
+  </si>
+  <si>
+    <t>diametros para tapas y envases de r28</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tapa 28 Seg. Corta </t>
+  </si>
+  <si>
+    <t>Tapa 28 Seg. Corta</t>
+  </si>
+  <si>
+    <t>Natural</t>
+  </si>
+  <si>
+    <t>Verde Oscuro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tapa 28 Seg. Linerless </t>
+  </si>
+  <si>
+    <t>Tapa 28 Seg. Linerless</t>
+  </si>
+  <si>
+    <t>Tapa 28 Seguridad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tapa 28 Seguridad </t>
+  </si>
+  <si>
+    <t>Azul Claro</t>
+  </si>
+  <si>
+    <t>Dorado</t>
+  </si>
+  <si>
+    <t>Rojo</t>
+  </si>
+  <si>
+    <t>Verde Claro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tapa 28 Seguridad  </t>
+  </si>
+  <si>
+    <t>seg corta</t>
+  </si>
+  <si>
+    <t>seg linerless</t>
+  </si>
+  <si>
+    <t>seguridad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tapa Distop 28 </t>
+  </si>
+  <si>
+    <t>Negro</t>
+  </si>
+  <si>
+    <t>distop</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tapa Fliptop 28 </t>
+  </si>
+  <si>
+    <t>fliptop</t>
+  </si>
+  <si>
+    <t>Tapa Push Pull 28 Blanca</t>
+  </si>
+  <si>
+    <t>Tapa Push Pull 28 Dorada</t>
+  </si>
+  <si>
+    <t>Tapa Push Pull 28 Fucsia</t>
+  </si>
+  <si>
+    <t>Tapa Push Pull 28 Natural</t>
+  </si>
+  <si>
+    <t>Tapa Push Pull 28 Negra</t>
+  </si>
+  <si>
+    <t>Tapa Push Pull 28 Verde</t>
+  </si>
+  <si>
+    <t>Tapa Twist 28 Dorado</t>
+  </si>
+  <si>
+    <t>Tapa Twist 28 Natural</t>
+  </si>
+  <si>
+    <t>Tapa Twist 28 Negro</t>
+  </si>
+  <si>
+    <t>push pull</t>
+  </si>
+  <si>
+    <t>Twist</t>
   </si>
 </sst>
 </file>
@@ -813,11 +936,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8C05424C-CE67-F944-BD85-0A191E147F69}">
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="18.5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="32.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
@@ -906,6 +1029,17 @@
       </c>
       <c r="C8" t="s">
         <v>35</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A9">
+        <v>28</v>
+      </c>
+      <c r="B9" t="s">
+        <v>97</v>
+      </c>
+      <c r="C9" t="s">
+        <v>98</v>
       </c>
     </row>
   </sheetData>
@@ -916,10 +1050,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE254BD3-8238-3B48-A36D-51D53B6E884E}">
-  <dimension ref="A1:J14"/>
+  <dimension ref="A1:J56"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.6640625" customWidth="1"/>
     <col min="2" max="2" width="11" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="12.1640625" bestFit="1" customWidth="1"/>
   </cols>
@@ -1372,6 +1506,1350 @@
         <v>10</v>
       </c>
     </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A15" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="B15" t="s">
+        <v>35</v>
+      </c>
+      <c r="C15">
+        <v>12</v>
+      </c>
+      <c r="D15" s="1">
+        <v>100</v>
+      </c>
+      <c r="E15" s="2">
+        <v>75</v>
+      </c>
+      <c r="F15" s="3">
+        <v>75</v>
+      </c>
+      <c r="G15" s="4">
+        <v>50</v>
+      </c>
+      <c r="H15" s="4">
+        <v>1000</v>
+      </c>
+      <c r="I15" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="J15">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A16" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="B16" t="s">
+        <v>35</v>
+      </c>
+      <c r="C16">
+        <v>12</v>
+      </c>
+      <c r="D16" s="1">
+        <v>100</v>
+      </c>
+      <c r="E16" s="2">
+        <v>75</v>
+      </c>
+      <c r="F16" s="3">
+        <v>75</v>
+      </c>
+      <c r="G16" s="4">
+        <v>50</v>
+      </c>
+      <c r="H16" s="4">
+        <v>1000</v>
+      </c>
+      <c r="I16" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="J16">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A17" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="B17" t="s">
+        <v>112</v>
+      </c>
+      <c r="C17">
+        <v>28</v>
+      </c>
+      <c r="D17" s="1">
+        <v>100</v>
+      </c>
+      <c r="E17" s="2">
+        <v>100</v>
+      </c>
+      <c r="F17" s="3">
+        <v>80</v>
+      </c>
+      <c r="G17" s="4">
+        <v>60</v>
+      </c>
+      <c r="H17" s="4">
+        <v>6500</v>
+      </c>
+      <c r="I17" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="J17">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A18" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="B18" t="s">
+        <v>112</v>
+      </c>
+      <c r="C18">
+        <v>28</v>
+      </c>
+      <c r="D18" s="1">
+        <v>100</v>
+      </c>
+      <c r="E18" s="2">
+        <v>100</v>
+      </c>
+      <c r="F18" s="3">
+        <v>80</v>
+      </c>
+      <c r="G18" s="4">
+        <v>60</v>
+      </c>
+      <c r="H18" s="4">
+        <v>6500</v>
+      </c>
+      <c r="I18" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="J18">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A19" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="B19" t="s">
+        <v>112</v>
+      </c>
+      <c r="C19">
+        <v>28</v>
+      </c>
+      <c r="D19" s="1">
+        <v>100</v>
+      </c>
+      <c r="E19" s="2">
+        <v>100</v>
+      </c>
+      <c r="F19" s="3">
+        <v>80</v>
+      </c>
+      <c r="G19" s="4">
+        <v>60</v>
+      </c>
+      <c r="H19" s="4">
+        <v>6500</v>
+      </c>
+      <c r="I19" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="J19">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A20" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="B20" t="s">
+        <v>112</v>
+      </c>
+      <c r="C20">
+        <v>28</v>
+      </c>
+      <c r="D20" s="1">
+        <v>100</v>
+      </c>
+      <c r="E20" s="2">
+        <v>100</v>
+      </c>
+      <c r="F20" s="3">
+        <v>80</v>
+      </c>
+      <c r="G20" s="4">
+        <v>60</v>
+      </c>
+      <c r="H20" s="4">
+        <v>6500</v>
+      </c>
+      <c r="I20" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="J20">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A21" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="B21" t="s">
+        <v>112</v>
+      </c>
+      <c r="C21">
+        <v>28</v>
+      </c>
+      <c r="D21" s="1">
+        <v>100</v>
+      </c>
+      <c r="E21" s="2">
+        <v>100</v>
+      </c>
+      <c r="F21" s="3">
+        <v>80</v>
+      </c>
+      <c r="G21" s="4">
+        <v>60</v>
+      </c>
+      <c r="H21" s="4">
+        <v>6500</v>
+      </c>
+      <c r="I21" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="J21">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A22" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="B22" t="s">
+        <v>112</v>
+      </c>
+      <c r="C22">
+        <v>28</v>
+      </c>
+      <c r="D22" s="1">
+        <v>100</v>
+      </c>
+      <c r="E22" s="2">
+        <v>100</v>
+      </c>
+      <c r="F22" s="3">
+        <v>80</v>
+      </c>
+      <c r="G22" s="4">
+        <v>60</v>
+      </c>
+      <c r="H22" s="4">
+        <v>6500</v>
+      </c>
+      <c r="I22" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="J22">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A23" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="B23" t="s">
+        <v>112</v>
+      </c>
+      <c r="C23">
+        <v>28</v>
+      </c>
+      <c r="D23" s="1">
+        <v>100</v>
+      </c>
+      <c r="E23" s="2">
+        <v>100</v>
+      </c>
+      <c r="F23" s="3">
+        <v>80</v>
+      </c>
+      <c r="G23" s="4">
+        <v>60</v>
+      </c>
+      <c r="H23" s="4">
+        <v>6500</v>
+      </c>
+      <c r="I23" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="J23">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A24" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="B24" t="s">
+        <v>113</v>
+      </c>
+      <c r="C24">
+        <v>28</v>
+      </c>
+      <c r="D24" s="1">
+        <v>100</v>
+      </c>
+      <c r="E24" s="2">
+        <v>100</v>
+      </c>
+      <c r="F24" s="3">
+        <v>80</v>
+      </c>
+      <c r="G24" s="4">
+        <v>65</v>
+      </c>
+      <c r="H24" s="4">
+        <v>6000</v>
+      </c>
+      <c r="I24" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="J24">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A25" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="B25" t="s">
+        <v>113</v>
+      </c>
+      <c r="C25">
+        <v>28</v>
+      </c>
+      <c r="D25" s="1">
+        <v>100</v>
+      </c>
+      <c r="E25" s="2">
+        <v>100</v>
+      </c>
+      <c r="F25" s="3">
+        <v>80</v>
+      </c>
+      <c r="G25" s="4">
+        <v>65</v>
+      </c>
+      <c r="H25" s="4">
+        <v>6000</v>
+      </c>
+      <c r="I25" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="J25">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A26" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="B26" t="s">
+        <v>113</v>
+      </c>
+      <c r="C26">
+        <v>28</v>
+      </c>
+      <c r="D26" s="1">
+        <v>100</v>
+      </c>
+      <c r="E26" s="2">
+        <v>100</v>
+      </c>
+      <c r="F26" s="3">
+        <v>80</v>
+      </c>
+      <c r="G26" s="4">
+        <v>65</v>
+      </c>
+      <c r="H26" s="4">
+        <v>6000</v>
+      </c>
+      <c r="I26" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="J26">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A27" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="B27" t="s">
+        <v>114</v>
+      </c>
+      <c r="C27">
+        <v>28</v>
+      </c>
+      <c r="D27" s="1">
+        <v>100</v>
+      </c>
+      <c r="E27" s="2">
+        <v>100</v>
+      </c>
+      <c r="F27" s="3">
+        <v>80</v>
+      </c>
+      <c r="G27" s="4">
+        <v>70</v>
+      </c>
+      <c r="H27" s="4">
+        <v>4000</v>
+      </c>
+      <c r="I27" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="J27">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A28" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="B28" t="s">
+        <v>114</v>
+      </c>
+      <c r="C28">
+        <v>28</v>
+      </c>
+      <c r="D28" s="1">
+        <v>100</v>
+      </c>
+      <c r="E28" s="2">
+        <v>100</v>
+      </c>
+      <c r="F28" s="3">
+        <v>80</v>
+      </c>
+      <c r="G28" s="4">
+        <v>70</v>
+      </c>
+      <c r="H28" s="4">
+        <v>4000</v>
+      </c>
+      <c r="I28" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="J28">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A29" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B29" t="s">
+        <v>114</v>
+      </c>
+      <c r="C29">
+        <v>28</v>
+      </c>
+      <c r="D29" s="1">
+        <v>100</v>
+      </c>
+      <c r="E29" s="2">
+        <v>100</v>
+      </c>
+      <c r="F29" s="3">
+        <v>80</v>
+      </c>
+      <c r="G29" s="4">
+        <v>70</v>
+      </c>
+      <c r="H29" s="4">
+        <v>4000</v>
+      </c>
+      <c r="I29" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="J29">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A30" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B30" t="s">
+        <v>114</v>
+      </c>
+      <c r="C30">
+        <v>28</v>
+      </c>
+      <c r="D30" s="1">
+        <v>100</v>
+      </c>
+      <c r="E30" s="2">
+        <v>100</v>
+      </c>
+      <c r="F30" s="3">
+        <v>80</v>
+      </c>
+      <c r="G30" s="4">
+        <v>70</v>
+      </c>
+      <c r="H30" s="4">
+        <v>4000</v>
+      </c>
+      <c r="I30" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="J30">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A31" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B31" t="s">
+        <v>114</v>
+      </c>
+      <c r="C31">
+        <v>28</v>
+      </c>
+      <c r="D31" s="1">
+        <v>100</v>
+      </c>
+      <c r="E31" s="2">
+        <v>100</v>
+      </c>
+      <c r="F31" s="3">
+        <v>80</v>
+      </c>
+      <c r="G31" s="4">
+        <v>70</v>
+      </c>
+      <c r="H31" s="4">
+        <v>4000</v>
+      </c>
+      <c r="I31" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="J31">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A32" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B32" t="s">
+        <v>114</v>
+      </c>
+      <c r="C32">
+        <v>28</v>
+      </c>
+      <c r="D32" s="1">
+        <v>100</v>
+      </c>
+      <c r="E32" s="2">
+        <v>100</v>
+      </c>
+      <c r="F32" s="3">
+        <v>80</v>
+      </c>
+      <c r="G32" s="4">
+        <v>70</v>
+      </c>
+      <c r="H32" s="4">
+        <v>4000</v>
+      </c>
+      <c r="I32" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="J32">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A33" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B33" t="s">
+        <v>114</v>
+      </c>
+      <c r="C33">
+        <v>28</v>
+      </c>
+      <c r="D33" s="1">
+        <v>100</v>
+      </c>
+      <c r="E33" s="2">
+        <v>100</v>
+      </c>
+      <c r="F33" s="3">
+        <v>80</v>
+      </c>
+      <c r="G33" s="4">
+        <v>70</v>
+      </c>
+      <c r="H33" s="4">
+        <v>4000</v>
+      </c>
+      <c r="I33" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="J33">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A34" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B34" t="s">
+        <v>114</v>
+      </c>
+      <c r="C34">
+        <v>28</v>
+      </c>
+      <c r="D34" s="1">
+        <v>100</v>
+      </c>
+      <c r="E34" s="2">
+        <v>100</v>
+      </c>
+      <c r="F34" s="3">
+        <v>80</v>
+      </c>
+      <c r="G34" s="4">
+        <v>70</v>
+      </c>
+      <c r="H34" s="4">
+        <v>4000</v>
+      </c>
+      <c r="I34" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="J34">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A35" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B35" t="s">
+        <v>114</v>
+      </c>
+      <c r="C35">
+        <v>28</v>
+      </c>
+      <c r="D35" s="1">
+        <v>100</v>
+      </c>
+      <c r="E35" s="2">
+        <v>100</v>
+      </c>
+      <c r="F35" s="3">
+        <v>80</v>
+      </c>
+      <c r="G35" s="4">
+        <v>70</v>
+      </c>
+      <c r="H35" s="4">
+        <v>4000</v>
+      </c>
+      <c r="I35" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="J35">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A36" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B36" t="s">
+        <v>114</v>
+      </c>
+      <c r="C36">
+        <v>28</v>
+      </c>
+      <c r="D36" s="1">
+        <v>100</v>
+      </c>
+      <c r="E36" s="2">
+        <v>100</v>
+      </c>
+      <c r="F36" s="3">
+        <v>80</v>
+      </c>
+      <c r="G36" s="4">
+        <v>70</v>
+      </c>
+      <c r="H36" s="4">
+        <v>4000</v>
+      </c>
+      <c r="I36" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="J36">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A37" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B37" t="s">
+        <v>114</v>
+      </c>
+      <c r="C37">
+        <v>28</v>
+      </c>
+      <c r="D37" s="1">
+        <v>100</v>
+      </c>
+      <c r="E37" s="2">
+        <v>100</v>
+      </c>
+      <c r="F37" s="3">
+        <v>80</v>
+      </c>
+      <c r="G37" s="4">
+        <v>70</v>
+      </c>
+      <c r="H37" s="4">
+        <v>4000</v>
+      </c>
+      <c r="I37" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="J37">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A38" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B38" t="s">
+        <v>114</v>
+      </c>
+      <c r="C38">
+        <v>28</v>
+      </c>
+      <c r="D38" s="1">
+        <v>100</v>
+      </c>
+      <c r="E38" s="2">
+        <v>100</v>
+      </c>
+      <c r="F38" s="3">
+        <v>80</v>
+      </c>
+      <c r="G38" s="4">
+        <v>70</v>
+      </c>
+      <c r="H38" s="4">
+        <v>4000</v>
+      </c>
+      <c r="I38" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="J38">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A39" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B39" t="s">
+        <v>114</v>
+      </c>
+      <c r="C39">
+        <v>28</v>
+      </c>
+      <c r="D39" s="1">
+        <v>100</v>
+      </c>
+      <c r="E39" s="2">
+        <v>100</v>
+      </c>
+      <c r="F39" s="3">
+        <v>80</v>
+      </c>
+      <c r="G39" s="4">
+        <v>70</v>
+      </c>
+      <c r="H39" s="4">
+        <v>4000</v>
+      </c>
+      <c r="I39" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="J39">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A40" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="B40" t="s">
+        <v>114</v>
+      </c>
+      <c r="C40">
+        <v>28</v>
+      </c>
+      <c r="D40" s="1">
+        <v>100</v>
+      </c>
+      <c r="E40" s="2">
+        <v>100</v>
+      </c>
+      <c r="F40" s="3">
+        <v>80</v>
+      </c>
+      <c r="G40" s="4">
+        <v>70</v>
+      </c>
+      <c r="H40" s="4">
+        <v>4000</v>
+      </c>
+      <c r="I40" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="J40">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A41" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="B41" t="s">
+        <v>117</v>
+      </c>
+      <c r="C41">
+        <v>28</v>
+      </c>
+      <c r="D41" s="1">
+        <v>400</v>
+      </c>
+      <c r="E41" s="2">
+        <v>380</v>
+      </c>
+      <c r="F41" s="3">
+        <v>350</v>
+      </c>
+      <c r="G41" s="4">
+        <v>350</v>
+      </c>
+      <c r="H41" s="4">
+        <v>500</v>
+      </c>
+      <c r="I41" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="J41">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A42" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="B42" t="s">
+        <v>117</v>
+      </c>
+      <c r="C42">
+        <v>28</v>
+      </c>
+      <c r="D42" s="1">
+        <v>400</v>
+      </c>
+      <c r="E42" s="2">
+        <v>380</v>
+      </c>
+      <c r="F42" s="3">
+        <v>350</v>
+      </c>
+      <c r="G42" s="4">
+        <v>350</v>
+      </c>
+      <c r="H42" s="4">
+        <v>500</v>
+      </c>
+      <c r="I42" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="J42">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="43" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A43" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="B43" t="s">
+        <v>117</v>
+      </c>
+      <c r="C43">
+        <v>28</v>
+      </c>
+      <c r="D43" s="1">
+        <v>400</v>
+      </c>
+      <c r="E43" s="2">
+        <v>380</v>
+      </c>
+      <c r="F43" s="3">
+        <v>350</v>
+      </c>
+      <c r="G43" s="4">
+        <v>350</v>
+      </c>
+      <c r="H43" s="4">
+        <v>500</v>
+      </c>
+      <c r="I43" s="5" t="s">
+        <v>116</v>
+      </c>
+      <c r="J43">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="44" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A44" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="B44" t="s">
+        <v>117</v>
+      </c>
+      <c r="C44">
+        <v>28</v>
+      </c>
+      <c r="D44" s="1">
+        <v>400</v>
+      </c>
+      <c r="E44" s="2">
+        <v>380</v>
+      </c>
+      <c r="F44" s="3">
+        <v>350</v>
+      </c>
+      <c r="G44" s="4">
+        <v>350</v>
+      </c>
+      <c r="H44" s="4">
+        <v>500</v>
+      </c>
+      <c r="I44" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="J44">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="45" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A45" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="B45" t="s">
+        <v>119</v>
+      </c>
+      <c r="C45">
+        <v>28</v>
+      </c>
+      <c r="D45" s="1">
+        <v>350</v>
+      </c>
+      <c r="E45" s="2">
+        <v>300</v>
+      </c>
+      <c r="F45" s="3">
+        <v>250</v>
+      </c>
+      <c r="G45" s="4">
+        <v>215</v>
+      </c>
+      <c r="H45" s="4">
+        <v>500</v>
+      </c>
+      <c r="I45" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="J45">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A46" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="B46" t="s">
+        <v>119</v>
+      </c>
+      <c r="C46">
+        <v>28</v>
+      </c>
+      <c r="D46" s="1">
+        <v>350</v>
+      </c>
+      <c r="E46" s="2">
+        <v>300</v>
+      </c>
+      <c r="F46" s="3">
+        <v>250</v>
+      </c>
+      <c r="G46" s="4">
+        <v>215</v>
+      </c>
+      <c r="H46" s="4">
+        <v>500</v>
+      </c>
+      <c r="I46" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="J46">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A47" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="B47" t="s">
+        <v>119</v>
+      </c>
+      <c r="C47">
+        <v>28</v>
+      </c>
+      <c r="D47" s="1">
+        <v>350</v>
+      </c>
+      <c r="E47" s="2">
+        <v>300</v>
+      </c>
+      <c r="F47" s="3">
+        <v>250</v>
+      </c>
+      <c r="G47" s="4">
+        <v>215</v>
+      </c>
+      <c r="H47" s="4">
+        <v>500</v>
+      </c>
+      <c r="I47" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="J47">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="48" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A48" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="B48" t="s">
+        <v>129</v>
+      </c>
+      <c r="C48">
+        <v>28</v>
+      </c>
+      <c r="D48" s="1">
+        <v>450</v>
+      </c>
+      <c r="E48" s="2">
+        <v>400</v>
+      </c>
+      <c r="F48" s="3">
+        <v>350</v>
+      </c>
+      <c r="G48" s="4">
+        <v>315</v>
+      </c>
+      <c r="H48" s="4">
+        <v>500</v>
+      </c>
+      <c r="I48" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="J48">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="49" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A49" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="B49" t="s">
+        <v>129</v>
+      </c>
+      <c r="C49">
+        <v>28</v>
+      </c>
+      <c r="D49" s="1">
+        <v>450</v>
+      </c>
+      <c r="E49" s="2">
+        <v>400</v>
+      </c>
+      <c r="F49" s="3">
+        <v>350</v>
+      </c>
+      <c r="G49" s="4">
+        <v>315</v>
+      </c>
+      <c r="H49" s="4">
+        <v>500</v>
+      </c>
+      <c r="I49" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="J49">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="50" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A50" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="B50" t="s">
+        <v>129</v>
+      </c>
+      <c r="C50">
+        <v>28</v>
+      </c>
+      <c r="D50" s="1">
+        <v>450</v>
+      </c>
+      <c r="E50" s="2">
+        <v>400</v>
+      </c>
+      <c r="F50" s="3">
+        <v>350</v>
+      </c>
+      <c r="G50" s="4">
+        <v>315</v>
+      </c>
+      <c r="H50" s="4">
+        <v>500</v>
+      </c>
+      <c r="I50" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="J50">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="51" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A51" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="B51" t="s">
+        <v>129</v>
+      </c>
+      <c r="C51">
+        <v>28</v>
+      </c>
+      <c r="D51" s="1">
+        <v>450</v>
+      </c>
+      <c r="E51" s="2">
+        <v>400</v>
+      </c>
+      <c r="F51" s="3">
+        <v>350</v>
+      </c>
+      <c r="G51" s="4">
+        <v>315</v>
+      </c>
+      <c r="H51" s="4">
+        <v>500</v>
+      </c>
+      <c r="I51" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="J51">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="52" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A52" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="B52" t="s">
+        <v>129</v>
+      </c>
+      <c r="C52">
+        <v>28</v>
+      </c>
+      <c r="D52" s="1">
+        <v>450</v>
+      </c>
+      <c r="E52" s="2">
+        <v>400</v>
+      </c>
+      <c r="F52" s="3">
+        <v>350</v>
+      </c>
+      <c r="G52" s="4">
+        <v>315</v>
+      </c>
+      <c r="H52" s="4">
+        <v>500</v>
+      </c>
+      <c r="I52" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="J52">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A53" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="B53" t="s">
+        <v>129</v>
+      </c>
+      <c r="C53">
+        <v>28</v>
+      </c>
+      <c r="D53" s="1">
+        <v>450</v>
+      </c>
+      <c r="E53" s="2">
+        <v>400</v>
+      </c>
+      <c r="F53" s="3">
+        <v>350</v>
+      </c>
+      <c r="G53" s="4">
+        <v>315</v>
+      </c>
+      <c r="H53" s="4">
+        <v>500</v>
+      </c>
+      <c r="I53" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="J53">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A54" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="B54" t="s">
+        <v>130</v>
+      </c>
+      <c r="C54">
+        <v>28</v>
+      </c>
+      <c r="D54" s="1">
+        <v>450</v>
+      </c>
+      <c r="E54" s="2">
+        <v>400</v>
+      </c>
+      <c r="F54" s="3">
+        <v>350</v>
+      </c>
+      <c r="G54" s="4">
+        <v>320</v>
+      </c>
+      <c r="H54" s="4">
+        <v>500</v>
+      </c>
+      <c r="I54" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="J54">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="55" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A55" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="B55" t="s">
+        <v>130</v>
+      </c>
+      <c r="C55">
+        <v>28</v>
+      </c>
+      <c r="D55" s="1">
+        <v>450</v>
+      </c>
+      <c r="E55" s="2">
+        <v>400</v>
+      </c>
+      <c r="F55" s="3">
+        <v>350</v>
+      </c>
+      <c r="G55" s="4">
+        <v>320</v>
+      </c>
+      <c r="H55" s="4">
+        <v>500</v>
+      </c>
+      <c r="I55" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="J55">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="56" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A56" s="6" t="s">
+        <v>128</v>
+      </c>
+      <c r="B56" t="s">
+        <v>130</v>
+      </c>
+      <c r="C56">
+        <v>28</v>
+      </c>
+      <c r="D56" s="1">
+        <v>450</v>
+      </c>
+      <c r="E56" s="2">
+        <v>400</v>
+      </c>
+      <c r="F56" s="3">
+        <v>350</v>
+      </c>
+      <c r="G56" s="4">
+        <v>320</v>
+      </c>
+      <c r="H56" s="4">
+        <v>500</v>
+      </c>
+      <c r="I56" s="5" t="s">
+        <v>116</v>
+      </c>
+      <c r="J56">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1379,14 +2857,15 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2DE0B0E3-6F34-0446-9ED2-DAECE5EB17B4}">
-  <dimension ref="A1:K19"/>
+  <dimension ref="A1:K22"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="2" width="21.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.83203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.6640625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="12.1640625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="13.83203125" customWidth="1"/>
     <col min="10" max="10" width="42.1640625" customWidth="1"/>
-    <col min="11" max="11" width="41" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="52.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.2">
@@ -1969,13 +3448,132 @@
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A19" s="10"/>
-      <c r="B19" s="10"/>
-      <c r="D19" s="11"/>
-      <c r="E19" s="12"/>
-      <c r="F19" s="13"/>
-      <c r="G19" s="14"/>
-      <c r="H19" s="14"/>
+      <c r="A19" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="C19">
+        <v>28</v>
+      </c>
+      <c r="D19" s="1">
+        <v>1350</v>
+      </c>
+      <c r="E19" s="2">
+        <v>1300</v>
+      </c>
+      <c r="F19" s="3">
+        <v>1267</v>
+      </c>
+      <c r="G19" s="4">
+        <v>1267</v>
+      </c>
+      <c r="H19" s="4">
+        <v>100</v>
+      </c>
+      <c r="I19">
+        <v>10</v>
+      </c>
+      <c r="J19" s="5" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A20" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="C20">
+        <v>28</v>
+      </c>
+      <c r="D20" s="1">
+        <v>1100</v>
+      </c>
+      <c r="E20" s="2">
+        <v>1050</v>
+      </c>
+      <c r="F20" s="3">
+        <v>1021</v>
+      </c>
+      <c r="G20" s="4">
+        <v>1021</v>
+      </c>
+      <c r="H20" s="4">
+        <v>100</v>
+      </c>
+      <c r="I20">
+        <v>10</v>
+      </c>
+      <c r="J20" s="5" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A21" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="C21">
+        <v>28</v>
+      </c>
+      <c r="D21" s="1">
+        <v>900</v>
+      </c>
+      <c r="E21" s="2">
+        <v>850</v>
+      </c>
+      <c r="F21" s="3">
+        <v>800</v>
+      </c>
+      <c r="G21" s="4">
+        <v>800</v>
+      </c>
+      <c r="H21" s="4">
+        <v>91</v>
+      </c>
+      <c r="I21">
+        <v>10</v>
+      </c>
+      <c r="J21" s="5" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A22" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="B22" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="C22">
+        <v>28</v>
+      </c>
+      <c r="D22" s="1">
+        <v>1050</v>
+      </c>
+      <c r="E22" s="2">
+        <v>1000</v>
+      </c>
+      <c r="F22" s="3">
+        <v>992</v>
+      </c>
+      <c r="G22" s="4">
+        <v>992</v>
+      </c>
+      <c r="H22" s="4">
+        <v>100</v>
+      </c>
+      <c r="I22">
+        <v>10</v>
+      </c>
+      <c r="J22" s="5" t="s">
+        <v>96</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>